<commit_message>
Publish retention activity-center filtering V1.1
</commit_message>
<xml_diff>
--- a/retention-activity/docs/保客活动号码级准入_功能清单.xlsx
+++ b/retention-activity/docs/保客活动号码级准入_功能清单.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能清单" sheetId="1" r:id="R09af31f2206c46e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验收场景" sheetId="2" r:id="Ra4384af715eb4fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待确认事项" sheetId="3" r:id="R6ea3cbdac9bd42e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能清单" sheetId="1" r:id="R1dbe64a07bd242fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="验收场景" sheetId="2" r:id="R9a5ce8fdaf914017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待确认事项" sheetId="3" r:id="R994c5fb5989e4654"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -178,6 +178,9 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -481,7 +484,7 @@
       <x:c r="A4" s="3"/>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="8" t="str">
-        <x:v>18项功能按三系统划分。完整规则、接口语义见配套需求文档。</x:v>
+        <x:v>18项功能含1项卡券中心既有能力。过滤改造由活动中心负责。</x:v>
       </x:c>
       <x:c r="D4" s="3"/>
       <x:c r="E4" s="3"/>
@@ -519,16 +522,16 @@
         <x:v>卡券中心</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>接收活动准入信息</x:v>
+        <x:v>沿用既有卡券查询接口</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
-        <x:v>活动关联卡券查询接口增加活动准入等级语义。号码级由卡券中心识别并执行过滤，正式字段名和枚举待对接。</x:v>
+        <x:v>现有接口已向活动中心提供业务场景、领取规则、核销方式等字段。本项为既有能力复用，本次无需新增卡券中心过滤接口或准入传参。</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>方向已确认，合同待确认</x:v>
+        <x:v>既有能力，用户已确认</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>S03；R08</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
         <x:v>AC21</x:v>
@@ -539,19 +542,19 @@
         <x:v>F02</x:v>
       </x:c>
       <x:c r="B7" s="21" t="str">
-        <x:v>卡券中心</x:v>
+        <x:v>活动中心后端</x:v>
       </x:c>
       <x:c r="C7" s="21" t="str">
         <x:v>按领取规则过滤</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
-        <x:v>号码级活动的全部查询场景仅返回领取规则为用户的卡券，与既有条件共同生效。</x:v>
+        <x:v>读取卡券中心返回的领取规则。号码级活动全部场景仅保留领取规则为用户的卡券，与既有关联条件共同生效。</x:v>
       </x:c>
       <x:c r="E7" s="21" t="str">
         <x:v>已确认</x:v>
       </x:c>
       <x:c r="F7" s="21" t="str">
-        <x:v>S01；R08</x:v>
+        <x:v>S01、S04；R08</x:v>
       </x:c>
       <x:c r="G7" s="21" t="str">
         <x:v>AC11、AC14、AC15</x:v>
@@ -562,19 +565,19 @@
         <x:v>F03</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
-        <x:v>卡券中心</x:v>
+        <x:v>活动中心后端</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
         <x:v>按业务场景过滤核销方式</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
-        <x:v>号码级且场景为BIMC（新）或维修保养（新）时，额外要求核销方式恰为线上核销。与用户领取规则为且。</x:v>
+        <x:v>读取卡券自身业务场景及核销方式。号码级且场景为BIMC（新）或维修保养（新）时，仅保留核销方式恰为线上核销的券，与用户领取规则为且。</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
         <x:v>已确认</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>S02；R09</x:v>
+        <x:v>S02、S04；R09</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
         <x:v>AC11—AC14、AC16</x:v>
@@ -585,19 +588,19 @@
         <x:v>F04</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>卡券中心</x:v>
+        <x:v>活动中心后端</x:v>
       </x:c>
       <x:c r="C9" s="21" t="str">
         <x:v>统一搜索与分页口径</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
-        <x:v>搜索、刷新、重置和翻页均保留准入过滤。建议在全部适用条件过滤后计算总数与分页。</x:v>
+        <x:v>搜索、刷新、重置和翻页持续应用号码级规则。建议由活动中心基于完整过滤结果计算总数与分页；既有接口分页的衔接方案见Q05。</x:v>
       </x:c>
       <x:c r="E9" s="21" t="str">
-        <x:v>规则已确认，分页实现建议</x:v>
+        <x:v>规则及责任已确认，分页方案待对齐</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
-        <x:v>S01、S02；R08、R09</x:v>
+        <x:v>S01、S02、S04；R08、R09</x:v>
       </x:c>
       <x:c r="G9" s="21" t="str">
         <x:v>AC17、AC19</x:v>
@@ -608,19 +611,19 @@
         <x:v>F05</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>卡券中心</x:v>
+        <x:v>活动中心后端</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>返回查询与校验信息</x:v>
+        <x:v>映射既有返回字段</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
-        <x:v>建议返回卡券标识、名称、业务场景、领取规则、核销方式及过滤后的分页信息，供展示和校验。</x:v>
+        <x:v>复用卡券中心已提供的场景、领取规则和核销方式，按既有接口的正式字段及枚举识别业务含义，供活动中心过滤及前端展示。</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>实现建议，合同待确认</x:v>
+        <x:v>字段已提供，映射待研发对齐</x:v>
       </x:c>
       <x:c r="F10" s="18" t="str">
-        <x:v>J01</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="G10" s="18" t="str">
         <x:v>AC21</x:v>
@@ -634,16 +637,16 @@
         <x:v>活动中心后端</x:v>
       </x:c>
       <x:c r="C11" s="21" t="str">
-        <x:v>传递准入查询上下文</x:v>
+        <x:v>保留活动准入查询上下文</x:v>
       </x:c>
       <x:c r="D11" s="21" t="str">
-        <x:v>调整管理后台与卡券中心对接，传递当前活动准入等级、业务场景及原搜索和分页条件。</x:v>
+        <x:v>接收管理后台的当前准入与查询条件，在活动中心保留准入供过滤使用。按既有合同调用卡券中心查询接口，无需向其新增传递准入等级。</x:v>
       </x:c>
       <x:c r="E11" s="21" t="str">
-        <x:v>方向已确认，合同待确认</x:v>
+        <x:v>责任已确认，对接细节待对齐</x:v>
       </x:c>
       <x:c r="F11" s="21" t="str">
-        <x:v>S03</x:v>
+        <x:v>S04</x:v>
       </x:c>
       <x:c r="G11" s="21" t="str">
         <x:v>AC17、AC21</x:v>
@@ -657,16 +660,16 @@
         <x:v>活动中心后端</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
-        <x:v>适配卡券中心返回结果</x:v>
+        <x:v>返回活动中心过滤结果</x:v>
       </x:c>
       <x:c r="D12" s="18" t="str">
-        <x:v>按正式合同映射返回字段和分页结果，向前端返回已过滤数据。不得补回本次被过滤的卡券。</x:v>
+        <x:v>活动中心执行F02、F03后向管理后台返回合规候选券，并按约定返回过滤后的总数与分页信息。不得补回已排除的卡券。</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>方向已确认，合同待确认</x:v>
+        <x:v>过滤责任已确认，分页方案待对齐</x:v>
       </x:c>
       <x:c r="F12" s="18" t="str">
-        <x:v>S03；R08、R09</x:v>
+        <x:v>S04；R08、R09</x:v>
       </x:c>
       <x:c r="G12" s="18" t="str">
         <x:v>AC11、AC21</x:v>
@@ -683,13 +686,13 @@
         <x:v>处理异常和旧调用兼容</x:v>
       </x:c>
       <x:c r="D13" s="21" t="str">
-        <x:v>需约定未传等级、未知枚举、历史草稿及接口异常的处理。建议号码级查询失败时提示重试，不降级到未过滤列表。</x:v>
+        <x:v>需约定管理后台未传等级、未知枚举、历史草稿及既有接口异常的处理。建议号码级查询失败时提示重试，不降级展示未过滤列表。</x:v>
       </x:c>
       <x:c r="E13" s="21" t="str">
-        <x:v>实现建议，合同待确认</x:v>
+        <x:v>实现建议，兼容策略待确认</x:v>
       </x:c>
       <x:c r="F13" s="21" t="str">
-        <x:v>J01</x:v>
+        <x:v>J01、S04</x:v>
       </x:c>
       <x:c r="G13" s="21" t="str">
         <x:v>AC22</x:v>
@@ -706,13 +709,13 @@
         <x:v>提交时复核已关联卡券</x:v>
       </x:c>
       <x:c r="D14" s="18" t="str">
-        <x:v>建议按当前准入及每张券自身场景复核领取规则和核销方式，避免等级切换、旧草稿或券配置变化绕过限制。</x:v>
+        <x:v>建议活动中心按当前准入及每张券自身场景复用过滤规则，避免等级切换、旧草稿或券配置变化绕过限制。复核触发时点与查询复用方式见Q06。</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>实现建议，责任待确认</x:v>
+        <x:v>实现建议，时点与范围待确认</x:v>
       </x:c>
       <x:c r="F14" s="18" t="str">
-        <x:v>J01</x:v>
+        <x:v>J01、S04</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
         <x:v>AC18、AC20</x:v>
@@ -867,13 +870,13 @@
         <x:v>联动关联卡券查询</x:v>
       </x:c>
       <x:c r="D21" s="21" t="str">
-        <x:v>step2选择卡券时携带当前准入与场景，搜索、重置、刷新、翻页继续携带。按服务返回结果展示候选券。</x:v>
+        <x:v>将当前准入、场景、搜索和分页条件提交给活动中心后端，搜索、重置、刷新、翻页保持当前准入。只展示活动中心过滤后的候选结果。</x:v>
       </x:c>
       <x:c r="E21" s="21" t="str">
-        <x:v>方向已确认，合同待确认</x:v>
+        <x:v>方向已确认，对接细节待对齐</x:v>
       </x:c>
       <x:c r="F21" s="21" t="str">
-        <x:v>S03；R08、R09</x:v>
+        <x:v>S04；R08、R09</x:v>
       </x:c>
       <x:c r="G21" s="21" t="str">
         <x:v>AC17、AC21</x:v>
@@ -931,7 +934,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3bbb78bb2944aa1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2766f952f48d4c19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1180,7 +1183,7 @@
         <x:v>号码级，分别查询两类场景，用户规则且仅线上核销</x:v>
       </x:c>
       <x:c r="D16" s="18" t="str">
-        <x:v>通过本次新增条件，仍需满足既有关联条件；可查询并关联。</x:v>
+        <x:v>活动中心保留并返回给管理后台；仍须满足既有关联条件，可查询、勾选并关联。</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
         <x:v>已确认规则</x:v>
@@ -1197,7 +1200,7 @@
         <x:v>号码级，两类场景，用户规则且线下或到店核销</x:v>
       </x:c>
       <x:c r="D17" s="21" t="str">
-        <x:v>不返回，不允许关联。</x:v>
+        <x:v>活动中心从接口返回数据中排除该券，不返回给管理后台，不允许关联。</x:v>
       </x:c>
       <x:c r="E17" s="21" t="str">
         <x:v>已确认规则</x:v>
@@ -1214,7 +1217,7 @@
         <x:v>号码级，两类场景，用户规则且组合、缺失或未知核销方式</x:v>
       </x:c>
       <x:c r="D18" s="18" t="str">
-        <x:v>均不等于线上核销，不放行。边界样本不代表正式接口枚举。</x:v>
+        <x:v>活动中心按精确值过滤，均不等于线上核销，不返回给管理后台。边界样本不代表正式接口枚举。</x:v>
       </x:c>
       <x:c r="E18" s="18" t="str">
         <x:v>精确匹配边界</x:v>
@@ -1231,7 +1234,7 @@
         <x:v>号码级，两类场景，VIN规则且线上核销</x:v>
       </x:c>
       <x:c r="D19" s="21" t="str">
-        <x:v>不满足用户规则，不返回，不允许关联。</x:v>
+        <x:v>活动中心判定不满足用户规则，排除该券，不返回给管理后台，不允许关联。</x:v>
       </x:c>
       <x:c r="E19" s="21" t="str">
         <x:v>已确认规则</x:v>
@@ -1282,10 +1285,10 @@
         <x:v>号码级执行券ID/名称搜索、重置、刷新、翻页</x:v>
       </x:c>
       <x:c r="D22" s="18" t="str">
-        <x:v>条件持续生效，无不合规券；建议总数和每页均基于完整过滤结果。</x:v>
+        <x:v>活动中心过滤条件持续生效，前端无不合规券；建议总数和分页均基于完整过滤结果。既有接口分页衔接见Q05。</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
-        <x:v>规则已确认，分页实现建议</x:v>
+        <x:v>规则及责任已确认，分页方案待对齐</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
@@ -1316,7 +1319,7 @@
         <x:v>号码级搜索无符合条件的券</x:v>
       </x:c>
       <x:c r="D24" s="18" t="str">
-        <x:v>建议返回空集合、总数0，前端显示无符合条件卡券。格式按正式合同。</x:v>
+        <x:v>建议活动中心返回空集合、总数0，前端显示无符合条件卡券；不得直接沿用过滤前总数。格式按两端约定。</x:v>
       </x:c>
       <x:c r="E24" s="18" t="str">
         <x:v>实现建议</x:v>
@@ -1333,7 +1336,7 @@
         <x:v>旧草稿恢复或选券后券配置变化再提交</x:v>
       </x:c>
       <x:c r="D25" s="21" t="str">
-        <x:v>建议按当前准入和券自身场景复核并拦截冲突，接口责任见Q06。</x:v>
+        <x:v>建议活动中心按当前准入和券自身场景复核并拦截冲突，触发时点与历史范围见Q06。</x:v>
       </x:c>
       <x:c r="E25" s="21" t="str">
         <x:v>实现建议</x:v>
@@ -1347,13 +1350,13 @@
         <x:v>F01、F05、F06、F07、F16</x:v>
       </x:c>
       <x:c r="C26" s="18" t="str">
-        <x:v>两系统用正式字段、枚举和分页数据联调</x:v>
+        <x:v>卡券中心既有接口返回场景、领取规则、核销方式，活动中心读取当前准入</x:v>
       </x:c>
       <x:c r="D26" s="18" t="str">
-        <x:v>活动准入与场景传递正确，结果与卡券中心过滤规则一致，无映射丢失。</x:v>
+        <x:v>既有字段映射正确，活动中心按R08、R09过滤并返回前端；无需新增卡券中心过滤接口或向其传入准入等级。</x:v>
       </x:c>
       <x:c r="E26" s="18" t="str">
-        <x:v>技术合同确定后执行</x:v>
+        <x:v>字段及责任已确认，联调待执行</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
@@ -1364,7 +1367,7 @@
         <x:v>F08</x:v>
       </x:c>
       <x:c r="C27" s="21" t="str">
-        <x:v>接口超时、未知枚举或旧调用未传准入</x:v>
+        <x:v>既有接口超时、未知枚举或管理后台旧调用未传准入</x:v>
       </x:c>
       <x:c r="D27" s="21" t="str">
         <x:v>按Q05约定处理；建议号码级失败不降级展示未过滤数据。</x:v>
@@ -1379,7 +1382,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6977a53c75b144b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc8f455d97a54514"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1421,7 +1424,7 @@
       <x:c r="A4" s="3"/>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="8" t="str">
-        <x:v>以下事项需在正式接口或交互评审中确定。</x:v>
+        <x:v>字段已提供、过滤责任已确认。以下仅列其余范围与实施细节。</x:v>
       </x:c>
       <x:c r="D4" s="3"/>
     </x:row>
@@ -1500,13 +1503,13 @@
         <x:v>Q05</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
-        <x:v>查询接口技术合同</x:v>
+        <x:v>既有字段映射与分页衔接</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>接口地址、方法、准入/场景/领取规则/核销方式正式字段及枚举、鉴权、分页、错误码与未传等级兼容。</x:v>
+        <x:v>字段已提供。需对齐既有正式字段与枚举映射、上游分页数据如何形成完整过滤结果及总数，以及活动中心异常和未传准入的兼容策略。</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
-        <x:v>卡券中心与活动中心后端</x:v>
+        <x:v>活动中心后端，卡券中心协助既有合同对齐</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
@@ -1517,10 +1520,10 @@
         <x:v>提交复核与历史数据</x:v>
       </x:c>
       <x:c r="C11" s="21" t="str">
-        <x:v>服务端复核接口由谁提供、何时调用，以及历史活动编辑/复制/草稿的兼容范围。</x:v>
+        <x:v>活动中心提交复核的触发时点、既有查询复用方式，以及历史活动编辑、复制、草稿的兼容范围。过滤责任已明确归活动中心。</x:v>
       </x:c>
       <x:c r="D11" s="21" t="str">
-        <x:v>产品与两端后端</x:v>
+        <x:v>产品与活动中心后端</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
@@ -1548,7 +1551,7 @@
         <x:v>本次精确线上核销限制仅点名BIMC（新）和维修保养（新）。其他同类场景如需扩展应补充明确清单。</x:v>
       </x:c>
       <x:c r="D13" s="21" t="str">
-        <x:v>产品与卡券中心</x:v>
+        <x:v>产品与活动中心后端</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1583,27 +1586,38 @@
         <x:v>S03</x:v>
       </x:c>
       <x:c r="B19" s="26" t="str">
-        <x:v>用户本次职责划分</x:v>
+        <x:v>初次职责讨论</x:v>
       </x:c>
       <x:c r="C19" s="26" t="str">
-        <x:v>卡券中心按准入与场景过滤，活动中心后端调整对接，管理后台调整位置及属性默认值。</x:v>
+        <x:v>管理后台位置及默认值调整仍有效；原卡券中心过滤分工已由S04替代，不作为当前实施依据。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="45" customHeight="1">
       <x:c r="A20" s="26" t="str">
+        <x:v>S04</x:v>
+      </x:c>
+      <x:c r="B20" s="26" t="str">
+        <x:v>用户最新职责确认</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="str">
+        <x:v>卡券中心已通过现有接口向活动中心提供所需字段，由活动中心过滤即可。本次不要求新增卡券中心过滤能力。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="45" customHeight="1">
+      <x:c r="A21" s="27" t="str">
         <x:v>J01</x:v>
       </x:c>
-      <x:c r="B20" s="26" t="str">
+      <x:c r="B21" s="27" t="str">
         <x:v>本次评审建议</x:v>
       </x:c>
-      <x:c r="C20" s="26" t="str">
-        <x:v>分页顺序、返回信息、提交复核、异常兼容与旧选择处理；具体合同或策略待确认。</x:v>
+      <x:c r="C21" s="27" t="str">
+        <x:v>分页衔接、提交复核时点、异常兼容与旧选择处理；具体实施方案或交互策略待确认。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R791638094e784cd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2078dedcb453409f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>